<commit_message>
feat: change graph ui
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57c0a2f26e30c5e3/Desktop/bigbrainblockchain3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="11_41ED09D99365140E62355476585DCE3A874741EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D691017F-0459-45D4-9E07-37CEF42EF816}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_41ED09D99365140E62355476585DCE3A874741EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE58BA6D-F351-40FF-8F26-CF97AB5F372B}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17625" yWindow="2235" windowWidth="11145" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="transactions" sheetId="1" r:id="rId1"/>
@@ -982,30 +982,15 @@
     <t>13.64</t>
   </si>
   <si>
-    <t>splits</t>
-  </si>
-  <si>
-    <t>li</t>
-  </si>
-  <si>
     <t>Italian Tomato Dinner</t>
   </si>
   <si>
     <t>15% Tips (tip On Total Bill); li's Bday Celebration</t>
   </si>
   <si>
-    <t>lin</t>
-  </si>
-  <si>
     <t>Even Split Between 5</t>
   </si>
   <si>
-    <t>lin:26.96</t>
-  </si>
-  <si>
-    <t>li:9.50</t>
-  </si>
-  <si>
     <t>Even Split Between 6</t>
   </si>
   <si>
@@ -1015,9 +1000,6 @@
     <t>lin &amp; li</t>
   </si>
   <si>
-    <t>li:27.28,lin:22.89</t>
-  </si>
-  <si>
     <t>Even Split Between 4</t>
   </si>
   <si>
@@ -1036,18 +1018,12 @@
     <t>15% Tips After Tax; Even Split</t>
   </si>
   <si>
-    <t>li:26.20</t>
-  </si>
-  <si>
     <t>15% Tips After Tax; Split 6 Ways</t>
   </si>
   <si>
     <t>Cypress Coach lines</t>
   </si>
   <si>
-    <t>li:6.79</t>
-  </si>
-  <si>
     <t>Lucky 9 Lanes Bowling</t>
   </si>
   <si>
@@ -1057,96 +1033,21 @@
     <t>Bowling</t>
   </si>
   <si>
-    <t>deng</t>
-  </si>
-  <si>
-    <t>deng:8.00</t>
-  </si>
-  <si>
-    <t>deng:6.00</t>
-  </si>
-  <si>
-    <t>deng:13.43</t>
-  </si>
-  <si>
-    <t>deng:11.20</t>
-  </si>
-  <si>
-    <t>deng:24.63,li:42.55</t>
-  </si>
-  <si>
-    <t>deng:14.33,li:14.33,lin:14.34</t>
-  </si>
-  <si>
-    <t>deng:10.74</t>
-  </si>
-  <si>
-    <t>deng:12.64,lin:14.45</t>
-  </si>
-  <si>
-    <t>deng:2.23,li:6.69</t>
-  </si>
-  <si>
-    <t>deng:23.33,li:23.33,lin:23.34</t>
-  </si>
-  <si>
-    <t>deng:13.02</t>
-  </si>
-  <si>
-    <t>deng:10.00,li:10.00</t>
-  </si>
-  <si>
-    <t>deng:17.36</t>
-  </si>
-  <si>
-    <t>deng:19.71,li:27.25,lin:27.24</t>
-  </si>
-  <si>
     <t>43% deng 57% li</t>
   </si>
   <si>
-    <t>deng:61.64,li:82.10</t>
-  </si>
-  <si>
-    <t>deng:22.67,lin:11.33</t>
-  </si>
-  <si>
-    <t>deng:254.72</t>
-  </si>
-  <si>
-    <t>deng:13.64</t>
-  </si>
-  <si>
     <t>Gang Nam KBBQ Dinner</t>
   </si>
   <si>
     <t>Bill Evenly Split (deng, li. ng)</t>
   </si>
   <si>
-    <t>deng:31.00,li:31.00,ng:31.00</t>
-  </si>
-  <si>
-    <t>ng</t>
-  </si>
-  <si>
-    <t>deng:29.92,li:26.86,lin:20.93,ng:27.29</t>
-  </si>
-  <si>
-    <t>deng:16.84,li:27.13,lin:17.19,ng:15.64</t>
-  </si>
-  <si>
     <t>Drawing Tablet</t>
   </si>
   <si>
-    <t>ng:66.08</t>
-  </si>
-  <si>
     <t>Movie Parking</t>
   </si>
   <si>
-    <t>deng:20.83,li:38.58,ng:25.66</t>
-  </si>
-  <si>
     <t>Hiking Gas Money</t>
   </si>
   <si>
@@ -1183,15 +1084,6 @@
     <t>ng Back</t>
   </si>
   <si>
-    <t>ng:41.43</t>
-  </si>
-  <si>
-    <t>deng:13.90,li:13.90,lin:13.90,ng:13.90</t>
-  </si>
-  <si>
-    <t>deng:20.47,li:24.09,ng:20.46</t>
-  </si>
-  <si>
     <t>For The King II</t>
   </si>
   <si>
@@ -1201,9 +1093,6 @@
     <t>21.02 Tips; The Handwritings Are Terrible But It's 132.9 Before Tax And Tips</t>
   </si>
   <si>
-    <t>deng:21.37,li:34.81,ng:23.82</t>
-  </si>
-  <si>
     <t>Beckett Card Grading</t>
   </si>
   <si>
@@ -1213,280 +1102,391 @@
     <t>Stanley Park Parking</t>
   </si>
   <si>
-    <t>ng:13.63</t>
-  </si>
-  <si>
-    <t>deng:17.50,li:17.50,ng:17.50,sim:17.50</t>
-  </si>
-  <si>
-    <t>sim</t>
-  </si>
-  <si>
-    <t>deng:36.67,li:36.67,ng:34.36,sim:18.20</t>
-  </si>
-  <si>
-    <t>deng:1.08,li:1.08,lin:1.08,ng:1.08,sim:1.08</t>
-  </si>
-  <si>
-    <t>deng:7.66,li:7.66,lin:7.66,ng:7.66,sim:7.66</t>
-  </si>
-  <si>
     <t>sim Got His Drink Mixed In, Otherwise Even Split Between 5</t>
   </si>
   <si>
-    <t>ng:15.65,sim:14.79</t>
-  </si>
-  <si>
-    <t>deng:24.17,li:29.00,ng:24.17,sim:24.16</t>
-  </si>
-  <si>
-    <t>deng:19.56,li:24.15,lin:31.40,ng:19.56,sim:21.13</t>
-  </si>
-  <si>
-    <t>deng:7.28,li:7.28,ng:7.28,sim:7.28</t>
-  </si>
-  <si>
     <t>3 From ng, li, sim Each</t>
   </si>
   <si>
-    <t>li:3.00,ng:3.00,sim:3.00</t>
-  </si>
-  <si>
-    <t>deng:7.00,lin:7.00,ng:7.00,sim:7.00</t>
-  </si>
-  <si>
-    <t>deng:24.56,li:23.30,lin:20.78,ng:23.30,sim:23.28</t>
-  </si>
-  <si>
-    <t>deng:22.34,li:22.34,ng:21.13,sim:21.13</t>
-  </si>
-  <si>
-    <t>deng:6.00,li:6.00,ng:6.00,sim:6.00</t>
-  </si>
-  <si>
-    <t>deng:3.50,li:3.50,ng:3.50,sim:3.50</t>
-  </si>
-  <si>
-    <t>deng:21.67,li:25.30,ng:19.02,sim:25.35</t>
-  </si>
-  <si>
-    <t>deng:3.00,lin:3.00,sim:3.00</t>
-  </si>
-  <si>
-    <t>deng:24.06,li:26.99,ng:21.61,sim:24.54</t>
-  </si>
-  <si>
-    <t>deng:20.14,li:23.59,lin:20.14,sim:20.13</t>
-  </si>
-  <si>
     <t>sim's Treat***; 15% Mandatory Service Charge</t>
   </si>
   <si>
-    <t>deng:22.88,lin:22.88,ng:22.88,sim:22.89</t>
-  </si>
-  <si>
-    <t>deng:30.40,li:30.40,lin:30.40,sim:30.40</t>
-  </si>
-  <si>
-    <t>sim:7.91</t>
-  </si>
-  <si>
-    <t>deng:29.79,li:24.00,lin:23.31,ng:20.18,sim:25.60</t>
-  </si>
-  <si>
     <t>Everyone Except ng And sim</t>
   </si>
   <si>
-    <t>deng:13.33,lin:13.33,sim:13.34</t>
-  </si>
-  <si>
-    <t>deng:31.53,li:36.38,lin:37.53,ng:22.98,sim:32.75</t>
-  </si>
-  <si>
     <t>Mcdicks On sim</t>
   </si>
   <si>
-    <t>sim:47.82</t>
-  </si>
-  <si>
-    <t>deng:24.68,li:27.69,lin:3.01,ng:20.41,sim:19.21</t>
-  </si>
-  <si>
-    <t>deng:18.50,li:18.50,lin:18.50,ng:18.50,sim:18.50</t>
-  </si>
-  <si>
     <t>1hr15min Prorated; ng/sim/li/deng Split</t>
   </si>
   <si>
-    <t>deng:13.10,li:13.10,ng:13.10,sim:13.10</t>
-  </si>
-  <si>
     <t>sim/ng Even Split; No Reciept Because The Cashier Is Too Intimitating For sim To Ask</t>
   </si>
   <si>
-    <t>ng:24.00,sim:24.00</t>
-  </si>
-  <si>
-    <t>deng:72.80,li:72.80,lin:72.80,ng:72.80,sim:72.80</t>
-  </si>
-  <si>
     <t>Split 1: sim; Split 2: li; Split 3: ng; Split 4: deng; 102 In Cash</t>
   </si>
   <si>
-    <t>deng:24.21,li:30.56,ng:24.82,sim:22.41</t>
-  </si>
-  <si>
-    <t>li:22.75,ng:21.05,sim:56.20</t>
-  </si>
-  <si>
     <t>Split Among Everyone Except lin (paid By sim Online)</t>
   </si>
   <si>
     <t>Where's THE Receipt -sim</t>
   </si>
   <si>
-    <t>deng:19.95,sim:14.70</t>
-  </si>
-  <si>
-    <t>deng:11.02,li:11.02,lin:11.02,ng:11.02,yu:11.04</t>
-  </si>
-  <si>
-    <t>deng:11.89,li:11.89,lin:11.89,ng:11.89,sim:11.89,yu:11.91</t>
-  </si>
-  <si>
-    <t>deng:20.17,yu:20.16</t>
-  </si>
-  <si>
-    <t>yu</t>
-  </si>
-  <si>
-    <t>deng:48.74,li:48.74,lin:48.74,sim:48.74,yu:48.75</t>
-  </si>
-  <si>
-    <t>deng:34.84,li:34.84,ng:33.61,sim:33.61,yu:29.92</t>
-  </si>
-  <si>
-    <t>deng:15.73,li:15.73,ng:15.73,yu:15.71</t>
-  </si>
-  <si>
-    <t>deng:4.50,li:4.50,ng:4.50,yu:4.50</t>
-  </si>
-  <si>
-    <t>deng:4.06,lin:4.06,ng:4.06,yu:4.07</t>
-  </si>
-  <si>
-    <t>deng:28.36,lin:28.36,ng:28.36,yu:31.40</t>
-  </si>
-  <si>
-    <t>deng:26.67,li:26.67,lin:26.67,ng:26.67,sim:26.67,yu:26.65</t>
-  </si>
-  <si>
-    <t>deng:25.66,lin:22.34,ng:22.94,sim:26.20,yu:23.55</t>
-  </si>
-  <si>
-    <t>yu:98.71</t>
-  </si>
-  <si>
-    <t>deng:20.69,dong:20.69,li:20.69,lin:20.69,ng:20.69,sim:20.69</t>
-  </si>
-  <si>
-    <t>deng:37.13,dong:37.13,lin:49.03,ng:41.00</t>
-  </si>
-  <si>
-    <t>deng:15.04,dong:15.04,li:15.04,ng:15.04,sim:19.98</t>
-  </si>
-  <si>
-    <t>deng:1.00,dong:1.00,li:1.00,ng:1.00,sim:1.00</t>
-  </si>
-  <si>
-    <t>deng:6.00,dong:6.00,li:6.00,ng:6.00,sim:6.00</t>
-  </si>
-  <si>
-    <t>deng:22.61,dong:26.33,lin:22.61</t>
-  </si>
-  <si>
-    <t>deng:20.33,dong:20.33,li:20.33,lin:20.33,ng:20.33,sim:20.33,yu:20.35</t>
-  </si>
-  <si>
-    <t>dong</t>
-  </si>
-  <si>
-    <t>deng:1.40,dong:1.40,li:1.40,ng:1.40,sim:1.40</t>
-  </si>
-  <si>
-    <t>dong:30.00,li:21.60,lin:30.00,ng:30.00,sim:30.00</t>
-  </si>
-  <si>
-    <t>deng:46.20,dong:46.20,li:39.15,lin:46.20,ng:46.20,yu:46.18</t>
-  </si>
-  <si>
-    <t>deng:12.00,dong:24.00,li:24.00,ng:12.00</t>
-  </si>
-  <si>
-    <t>deng:18.45,dong:20.74,li:22.56,lin:19.78,ng:26.77</t>
-  </si>
-  <si>
-    <t>deng:17.01,dong:17.01,li:17.01,lin:17.01,yu:17.03</t>
-  </si>
-  <si>
-    <t>deng:16.38,dong:16.38,li:16.38,lin:16.38,yu:16.37</t>
-  </si>
-  <si>
-    <t>deng:5.88,dong:5.88,li:5.88,lin:5.88,yu:5.88</t>
-  </si>
-  <si>
-    <t>deng:2.80,dong:2.80</t>
-  </si>
-  <si>
-    <t>deng:5.91,dong:4.31,li:25.81,lin:11.40,ng:6.20,sim:190.61,yu:14.11</t>
-  </si>
-  <si>
-    <t>deng:1.64,dong:17.34,li:123.41,sim:38.46</t>
-  </si>
-  <si>
-    <t>deng:22.00,dong:22.00,li:22.00,sim:22.00</t>
-  </si>
-  <si>
-    <t>deng:10.13,dong:10.13,li:10.13,sim:10.11</t>
-  </si>
-  <si>
-    <t>deng:27.11,dong:22.00,li:35.88,lin:32.86,ng:30.13,sim:22.00,yu:41.21</t>
-  </si>
-  <si>
-    <t>deng:23.95,dong:23.95,lin:23.95,ng:23.95,sim:23.95,yu:23.94</t>
-  </si>
-  <si>
-    <t>deng:23.15,dong:23.15,li:23.15,lin:23.15,sim:23.15</t>
-  </si>
-  <si>
-    <t>deng:25.66,dong:11.47,li:29.58,lin:22.94,sim:22.89</t>
-  </si>
-  <si>
-    <t>deng:26.25,dong:27.02,li:30.48,lin:26.25</t>
-  </si>
-  <si>
-    <t>deng:37.98,dong:37.98,li:37.98,lin:37.98,ng:37.98,sim:37.98,yu:37.95</t>
-  </si>
-  <si>
-    <t>deng:25.88,dong:29.84,li:39.68,lin:18.69,ng:25.88,yu:20.70</t>
-  </si>
-  <si>
-    <t>deng:9.05,dong:9.05,li:9.05,lin:9.05,yu:9.07</t>
-  </si>
-  <si>
-    <t>deng:22.94,dong:22.94,li:22.94,ng:22.94,sim:22.95</t>
-  </si>
-  <si>
-    <t>deng:32.59,dong:32.59,li:37.10,ng:37.10,sim:32.59</t>
-  </si>
-  <si>
-    <t>deng:25.22,dong:22.93,li:28.97,ng:23.17,yu:27.87</t>
-  </si>
-  <si>
-    <t>deng:27.01,dong:24.93,li:27.90,ng:24.34,yu:25.82</t>
-  </si>
-  <si>
-    <t>deng:20.82,dong:20.82,li:20.82,ng:20.82,yu:20.82</t>
+    <t>spTimmyts</t>
+  </si>
+  <si>
+    <t>Timmy</t>
+  </si>
+  <si>
+    <t>Timmy:9.50</t>
+  </si>
+  <si>
+    <t>Timmy:26.20</t>
+  </si>
+  <si>
+    <t>Timmy:6.79</t>
+  </si>
+  <si>
+    <t>Leon</t>
+  </si>
+  <si>
+    <t>Leon:26.96</t>
+  </si>
+  <si>
+    <t>Timmy:27.28,Leon:22.89</t>
+  </si>
+  <si>
+    <t>Jayden</t>
+  </si>
+  <si>
+    <t>Jayden:66.08</t>
+  </si>
+  <si>
+    <t>Jayden:41.43</t>
+  </si>
+  <si>
+    <t>Jayden:13.63</t>
+  </si>
+  <si>
+    <t>Henry</t>
+  </si>
+  <si>
+    <t>Henry:98.71</t>
+  </si>
+  <si>
+    <t>Danny</t>
+  </si>
+  <si>
+    <t>Danny:8.00</t>
+  </si>
+  <si>
+    <t>Danny:6.00</t>
+  </si>
+  <si>
+    <t>Danny:13.43</t>
+  </si>
+  <si>
+    <t>Danny:11.20</t>
+  </si>
+  <si>
+    <t>Danny:24.63,Timmy:42.55</t>
+  </si>
+  <si>
+    <t>Danny:14.33,Timmy:14.33,Leon:14.34</t>
+  </si>
+  <si>
+    <t>Danny:10.74</t>
+  </si>
+  <si>
+    <t>Danny:12.64,Leon:14.45</t>
+  </si>
+  <si>
+    <t>Danny:2.23,Timmy:6.69</t>
+  </si>
+  <si>
+    <t>Danny:23.33,Timmy:23.33,Leon:23.34</t>
+  </si>
+  <si>
+    <t>Danny:13.02</t>
+  </si>
+  <si>
+    <t>Danny:10.00,Timmy:10.00</t>
+  </si>
+  <si>
+    <t>Danny:17.36</t>
+  </si>
+  <si>
+    <t>Danny:19.71,Timmy:27.25,Leon:27.24</t>
+  </si>
+  <si>
+    <t>Danny:61.64,Timmy:82.10</t>
+  </si>
+  <si>
+    <t>Danny:22.67,Leon:11.33</t>
+  </si>
+  <si>
+    <t>Danny:254.72</t>
+  </si>
+  <si>
+    <t>Danny:13.64</t>
+  </si>
+  <si>
+    <t>Danny:31.00,Timmy:31.00,Jayden:31.00</t>
+  </si>
+  <si>
+    <t>Danny:29.92,Timmy:26.86,Leon:20.93,Jayden:27.29</t>
+  </si>
+  <si>
+    <t>Danny:16.84,Timmy:27.13,Leon:17.19,Jayden:15.64</t>
+  </si>
+  <si>
+    <t>Danny:20.83,Timmy:38.58,Jayden:25.66</t>
+  </si>
+  <si>
+    <t>Danny:13.90,Timmy:13.90,Leon:13.90,Jayden:13.90</t>
+  </si>
+  <si>
+    <t>Danny:20.47,Timmy:24.09,Jayden:20.46</t>
+  </si>
+  <si>
+    <t>Danny:21.37,Timmy:34.81,Jayden:23.82</t>
+  </si>
+  <si>
+    <t>Danny:17.50,Timmy:17.50,Jayden:17.50,Calvin:17.50</t>
+  </si>
+  <si>
+    <t>Calvin</t>
+  </si>
+  <si>
+    <t>Danny:36.67,Timmy:36.67,Jayden:34.36,Calvin:18.20</t>
+  </si>
+  <si>
+    <t>Danny:1.08,Timmy:1.08,Leon:1.08,Jayden:1.08,Calvin:1.08</t>
+  </si>
+  <si>
+    <t>Danny:7.66,Timmy:7.66,Leon:7.66,Jayden:7.66,Calvin:7.66</t>
+  </si>
+  <si>
+    <t>Jayden:15.65,Calvin:14.79</t>
+  </si>
+  <si>
+    <t>Danny:24.17,Timmy:29.00,Jayden:24.17,Calvin:24.16</t>
+  </si>
+  <si>
+    <t>Danny:19.56,Timmy:24.15,Leon:31.40,Jayden:19.56,Calvin:21.13</t>
+  </si>
+  <si>
+    <t>Danny:7.28,Timmy:7.28,Jayden:7.28,Calvin:7.28</t>
+  </si>
+  <si>
+    <t>Timmy:3.00,Jayden:3.00,Calvin:3.00</t>
+  </si>
+  <si>
+    <t>Danny:7.00,Leon:7.00,Jayden:7.00,Calvin:7.00</t>
+  </si>
+  <si>
+    <t>Danny:24.56,Timmy:23.30,Leon:20.78,Jayden:23.30,Calvin:23.28</t>
+  </si>
+  <si>
+    <t>Danny:22.34,Timmy:22.34,Jayden:21.13,Calvin:21.13</t>
+  </si>
+  <si>
+    <t>Danny:6.00,Timmy:6.00,Jayden:6.00,Calvin:6.00</t>
+  </si>
+  <si>
+    <t>Danny:3.50,Timmy:3.50,Jayden:3.50,Calvin:3.50</t>
+  </si>
+  <si>
+    <t>Danny:21.67,Timmy:25.30,Jayden:19.02,Calvin:25.35</t>
+  </si>
+  <si>
+    <t>Danny:3.00,Leon:3.00,Calvin:3.00</t>
+  </si>
+  <si>
+    <t>Danny:24.06,Timmy:26.99,Jayden:21.61,Calvin:24.54</t>
+  </si>
+  <si>
+    <t>Danny:20.14,Timmy:23.59,Leon:20.14,Calvin:20.13</t>
+  </si>
+  <si>
+    <t>Danny:22.88,Leon:22.88,Jayden:22.88,Calvin:22.89</t>
+  </si>
+  <si>
+    <t>Danny:30.40,Timmy:30.40,Leon:30.40,Calvin:30.40</t>
+  </si>
+  <si>
+    <t>Calvin:7.91</t>
+  </si>
+  <si>
+    <t>Danny:29.79,Timmy:24.00,Leon:23.31,Jayden:20.18,Calvin:25.60</t>
+  </si>
+  <si>
+    <t>Danny:13.33,Leon:13.33,Calvin:13.34</t>
+  </si>
+  <si>
+    <t>Danny:31.53,Timmy:36.38,Leon:37.53,Jayden:22.98,Calvin:32.75</t>
+  </si>
+  <si>
+    <t>Calvin:47.82</t>
+  </si>
+  <si>
+    <t>Danny:24.68,Timmy:27.69,Leon:3.01,Jayden:20.41,Calvin:19.21</t>
+  </si>
+  <si>
+    <t>Danny:18.50,Timmy:18.50,Leon:18.50,Jayden:18.50,Calvin:18.50</t>
+  </si>
+  <si>
+    <t>Danny:13.10,Timmy:13.10,Jayden:13.10,Calvin:13.10</t>
+  </si>
+  <si>
+    <t>Jayden:24.00,Calvin:24.00</t>
+  </si>
+  <si>
+    <t>Danny:72.80,Timmy:72.80,Leon:72.80,Jayden:72.80,Calvin:72.80</t>
+  </si>
+  <si>
+    <t>Danny:24.21,Timmy:30.56,Jayden:24.82,Calvin:22.41</t>
+  </si>
+  <si>
+    <t>Timmy:22.75,Jayden:21.05,Calvin:56.20</t>
+  </si>
+  <si>
+    <t>Danny:19.95,Calvin:14.70</t>
+  </si>
+  <si>
+    <t>Danny:22.61,Andy:26.33,Leon:22.61</t>
+  </si>
+  <si>
+    <t>Andy</t>
+  </si>
+  <si>
+    <t>Danny:2.80,Andy:2.80</t>
+  </si>
+  <si>
+    <t>Danny:26.25,Andy:27.02,Timmy:30.48,Leon:26.25</t>
+  </si>
+  <si>
+    <t>Danny:37.13,Andy:37.13,Leon:49.03,Jayden:41.00</t>
+  </si>
+  <si>
+    <t>Danny:12.00,Andy:24.00,Timmy:24.00,Jayden:12.00</t>
+  </si>
+  <si>
+    <t>Danny:18.45,Andy:20.74,Timmy:22.56,Leon:19.78,Jayden:26.77</t>
+  </si>
+  <si>
+    <t>Danny:11.02,Timmy:11.02,Leon:11.02,Jayden:11.02,Henry:11.04</t>
+  </si>
+  <si>
+    <t>Danny:20.17,Henry:20.16</t>
+  </si>
+  <si>
+    <t>Danny:46.20,Andy:46.20,Timmy:39.15,Leon:46.20,Jayden:46.20,Henry:46.18</t>
+  </si>
+  <si>
+    <t>Danny:15.73,Timmy:15.73,Jayden:15.73,Henry:15.71</t>
+  </si>
+  <si>
+    <t>Danny:4.50,Timmy:4.50,Jayden:4.50,Henry:4.50</t>
+  </si>
+  <si>
+    <t>Danny:17.01,Andy:17.01,Timmy:17.01,Leon:17.01,Henry:17.03</t>
+  </si>
+  <si>
+    <t>Danny:16.38,Andy:16.38,Timmy:16.38,Leon:16.38,Henry:16.37</t>
+  </si>
+  <si>
+    <t>Danny:5.88,Andy:5.88,Timmy:5.88,Leon:5.88,Henry:5.88</t>
+  </si>
+  <si>
+    <t>Danny:4.06,Leon:4.06,Jayden:4.06,Henry:4.07</t>
+  </si>
+  <si>
+    <t>Danny:28.36,Leon:28.36,Jayden:28.36,Henry:31.40</t>
+  </si>
+  <si>
+    <t>Danny:25.88,Andy:29.84,Timmy:39.68,Leon:18.69,Jayden:25.88,Henry:20.70</t>
+  </si>
+  <si>
+    <t>Danny:9.05,Andy:9.05,Timmy:9.05,Leon:9.05,Henry:9.07</t>
+  </si>
+  <si>
+    <t>Danny:25.22,Andy:22.93,Timmy:28.97,Jayden:23.17,Henry:27.87</t>
+  </si>
+  <si>
+    <t>Danny:27.01,Andy:24.93,Timmy:27.90,Jayden:24.34,Henry:25.82</t>
+  </si>
+  <si>
+    <t>Danny:20.82,Andy:20.82,Timmy:20.82,Jayden:20.82,Henry:20.82</t>
+  </si>
+  <si>
+    <t>Danny:20.69,Andy:20.69,Timmy:20.69,Leon:20.69,Jayden:20.69,Calvin:20.69</t>
+  </si>
+  <si>
+    <t>Danny:15.04,Andy:15.04,Timmy:15.04,Jayden:15.04,Calvin:19.98</t>
+  </si>
+  <si>
+    <t>Danny:1.00,Andy:1.00,Timmy:1.00,Jayden:1.00,Calvin:1.00</t>
+  </si>
+  <si>
+    <t>Danny:6.00,Andy:6.00,Timmy:6.00,Jayden:6.00,Calvin:6.00</t>
+  </si>
+  <si>
+    <t>Danny:11.89,Timmy:11.89,Leon:11.89,Jayden:11.89,Calvin:11.89,Henry:11.91</t>
+  </si>
+  <si>
+    <t>Danny:20.33,Andy:20.33,Timmy:20.33,Leon:20.33,Jayden:20.33,Calvin:20.33,Henry:20.35</t>
+  </si>
+  <si>
+    <t>Danny:1.40,Andy:1.40,Timmy:1.40,Jayden:1.40,Calvin:1.40</t>
+  </si>
+  <si>
+    <t>Danny:48.74,Timmy:48.74,Leon:48.74,Calvin:48.74,Henry:48.75</t>
+  </si>
+  <si>
+    <t>Andy:30.00,Timmy:21.60,Leon:30.00,Jayden:30.00,Calvin:30.00</t>
+  </si>
+  <si>
+    <t>Danny:34.84,Timmy:34.84,Jayden:33.61,Calvin:33.61,Henry:29.92</t>
+  </si>
+  <si>
+    <t>Danny:5.91,Andy:4.31,Timmy:25.81,Leon:11.40,Jayden:6.20,Calvin:190.61,Henry:14.11</t>
+  </si>
+  <si>
+    <t>Danny:1.64,Andy:17.34,Timmy:123.41,Calvin:38.46</t>
+  </si>
+  <si>
+    <t>Danny:22.00,Andy:22.00,Timmy:22.00,Calvin:22.00</t>
+  </si>
+  <si>
+    <t>Danny:10.13,Andy:10.13,Timmy:10.13,Calvin:10.11</t>
+  </si>
+  <si>
+    <t>Danny:27.11,Andy:22.00,Timmy:35.88,Leon:32.86,Jayden:30.13,Calvin:22.00,Henry:41.21</t>
+  </si>
+  <si>
+    <t>Danny:23.95,Andy:23.95,Leon:23.95,Jayden:23.95,Calvin:23.95,Henry:23.94</t>
+  </si>
+  <si>
+    <t>Danny:23.15,Andy:23.15,Timmy:23.15,Leon:23.15,Calvin:23.15</t>
+  </si>
+  <si>
+    <t>Danny:25.66,Andy:11.47,Timmy:29.58,Leon:22.94,Calvin:22.89</t>
+  </si>
+  <si>
+    <t>Danny:37.98,Andy:37.98,Timmy:37.98,Leon:37.98,Jayden:37.98,Calvin:37.98,Henry:37.95</t>
+  </si>
+  <si>
+    <t>Danny:22.94,Andy:22.94,Timmy:22.94,Jayden:22.94,Calvin:22.95</t>
+  </si>
+  <si>
+    <t>Danny:32.59,Andy:32.59,Timmy:37.10,Jayden:37.10,Calvin:32.59</t>
+  </si>
+  <si>
+    <t>Danny:26.67,Timmy:26.67,Leon:26.67,Jayden:26.67,Calvin:26.67,Henry:26.65</t>
+  </si>
+  <si>
+    <t>Danny:25.66,Leon:22.34,Jayden:22.94,Calvin:26.20,Henry:23.55</t>
   </si>
 </sst>
 </file>
@@ -1870,7 +1870,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>320</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1878,19 +1878,19 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1898,19 +1898,19 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>365</v>
+        <v>338</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1918,19 +1918,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C4" t="s">
-        <v>366</v>
+        <v>339</v>
       </c>
       <c r="D4" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E4" t="s">
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>367</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1944,13 +1944,13 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>369</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1964,13 +1964,13 @@
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E6" t="s">
         <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1981,13 +1981,13 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>346</v>
+        <v>385</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1998,16 +1998,16 @@
         <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D8" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E8" t="s">
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2021,13 +2021,13 @@
         <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E9" t="s">
         <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>370</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2038,13 +2038,13 @@
         <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E10" t="s">
         <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2055,16 +2055,16 @@
         <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D11" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E11" t="s">
         <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2075,16 +2075,16 @@
         <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D12" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E12" t="s">
         <v>34</v>
       </c>
       <c r="F12" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2095,16 +2095,16 @@
         <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>403</v>
+        <v>360</v>
       </c>
       <c r="D13" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -2118,13 +2118,13 @@
         <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E14" t="s">
         <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2138,13 +2138,13 @@
         <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E15" t="s">
         <v>43</v>
       </c>
       <c r="F15" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2158,13 +2158,13 @@
         <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E16" t="s">
         <v>47</v>
       </c>
       <c r="F16" t="s">
-        <v>326</v>
+        <v>376</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -2175,13 +2175,13 @@
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E17" t="s">
         <v>49</v>
       </c>
       <c r="F17" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -2195,13 +2195,13 @@
         <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
       </c>
       <c r="F18" t="s">
-        <v>460</v>
+        <v>444</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2212,16 +2212,16 @@
         <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="D19" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E19" t="s">
         <v>56</v>
       </c>
       <c r="F19" t="s">
-        <v>443</v>
+        <v>470</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2229,19 +2229,19 @@
         <v>54</v>
       </c>
       <c r="B20" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C20" t="s">
         <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E20" t="s">
         <v>58</v>
       </c>
       <c r="F20" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -2252,13 +2252,13 @@
         <v>59</v>
       </c>
       <c r="D21" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E21" t="s">
         <v>60</v>
       </c>
       <c r="F21" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2269,16 +2269,16 @@
         <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D22" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E22" t="s">
         <v>61</v>
       </c>
       <c r="F22" t="s">
-        <v>331</v>
+        <v>377</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2286,19 +2286,19 @@
         <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C23" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="D23" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E23" t="s">
         <v>63</v>
       </c>
       <c r="F23" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2312,13 +2312,13 @@
         <v>66</v>
       </c>
       <c r="D24" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E24" t="s">
         <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2329,13 +2329,13 @@
         <v>68</v>
       </c>
       <c r="D25" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E25" t="s">
         <v>69</v>
       </c>
       <c r="F25" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2349,13 +2349,13 @@
         <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E26" t="s">
         <v>72</v>
       </c>
       <c r="F26" t="s">
-        <v>347</v>
+        <v>386</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2366,16 +2366,16 @@
         <v>74</v>
       </c>
       <c r="C27" t="s">
-        <v>371</v>
+        <v>340</v>
       </c>
       <c r="D27" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E27" t="s">
         <v>75</v>
       </c>
       <c r="F27" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2389,13 +2389,13 @@
         <v>78</v>
       </c>
       <c r="D28" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E28" t="s">
         <v>79</v>
       </c>
       <c r="F28" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2406,16 +2406,16 @@
         <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>408</v>
+        <v>361</v>
       </c>
       <c r="D29" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E29" t="s">
         <v>82</v>
       </c>
       <c r="F29" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2423,19 +2423,19 @@
         <v>80</v>
       </c>
       <c r="B30" t="s">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="C30" t="s">
         <v>83</v>
       </c>
       <c r="D30" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E30" t="s">
         <v>84</v>
       </c>
       <c r="F30" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2449,13 +2449,13 @@
         <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E31" t="s">
         <v>89</v>
       </c>
       <c r="F31" t="s">
-        <v>374</v>
+        <v>406</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2463,19 +2463,19 @@
         <v>90</v>
       </c>
       <c r="B32" t="s">
-        <v>375</v>
+        <v>342</v>
       </c>
       <c r="C32" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="D32" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E32" t="s">
         <v>91</v>
       </c>
       <c r="F32" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2483,19 +2483,19 @@
         <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>376</v>
+        <v>343</v>
       </c>
       <c r="C33" t="s">
         <v>92</v>
       </c>
       <c r="D33" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E33" t="s">
         <v>93</v>
       </c>
       <c r="F33" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2509,13 +2509,13 @@
         <v>96</v>
       </c>
       <c r="D34" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E34" t="s">
         <v>97</v>
       </c>
       <c r="F34" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2523,19 +2523,19 @@
         <v>98</v>
       </c>
       <c r="B35" t="s">
-        <v>375</v>
+        <v>342</v>
       </c>
       <c r="C35" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="D35" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E35" t="s">
         <v>99</v>
       </c>
       <c r="F35" t="s">
-        <v>413</v>
+        <v>423</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2546,13 +2546,13 @@
         <v>100</v>
       </c>
       <c r="D36" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E36" t="s">
         <v>101</v>
       </c>
       <c r="F36" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2566,13 +2566,13 @@
         <v>96</v>
       </c>
       <c r="D37" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E37" t="s">
         <v>103</v>
       </c>
       <c r="F37" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2586,13 +2586,13 @@
         <v>106</v>
       </c>
       <c r="D38" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E38" t="s">
         <v>107</v>
       </c>
       <c r="F38" t="s">
-        <v>446</v>
+        <v>473</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2606,13 +2606,13 @@
         <v>109</v>
       </c>
       <c r="D39" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E39" t="s">
         <v>82</v>
       </c>
       <c r="F39" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2620,19 +2620,19 @@
         <v>110</v>
       </c>
       <c r="B40" t="s">
-        <v>365</v>
+        <v>338</v>
       </c>
       <c r="C40" t="s">
         <v>111</v>
       </c>
       <c r="D40" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E40" t="s">
         <v>112</v>
       </c>
       <c r="F40" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2643,13 +2643,13 @@
         <v>114</v>
       </c>
       <c r="D41" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E41" t="s">
         <v>115</v>
       </c>
       <c r="F41" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2660,16 +2660,16 @@
         <v>117</v>
       </c>
       <c r="C42" t="s">
-        <v>377</v>
+        <v>344</v>
       </c>
       <c r="D42" t="s">
-        <v>462</v>
+        <v>445</v>
       </c>
       <c r="E42" t="s">
         <v>118</v>
       </c>
       <c r="F42" t="s">
-        <v>465</v>
+        <v>453</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2680,16 +2680,16 @@
         <v>120</v>
       </c>
       <c r="C43" t="s">
+        <v>345</v>
+      </c>
+      <c r="D43" t="s">
         <v>378</v>
-      </c>
-      <c r="D43" t="s">
-        <v>368</v>
       </c>
       <c r="E43" t="s">
         <v>121</v>
       </c>
       <c r="F43" t="s">
-        <v>348</v>
+        <v>387</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2700,16 +2700,16 @@
         <v>122</v>
       </c>
       <c r="C44" t="s">
-        <v>379</v>
+        <v>346</v>
       </c>
       <c r="D44" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E44" t="s">
         <v>123</v>
       </c>
       <c r="F44" t="s">
-        <v>349</v>
+        <v>388</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2723,13 +2723,13 @@
         <v>126</v>
       </c>
       <c r="D45" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E45" t="s">
         <v>127</v>
       </c>
       <c r="F45" t="s">
-        <v>466</v>
+        <v>449</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2740,16 +2740,16 @@
         <v>129</v>
       </c>
       <c r="C46" t="s">
-        <v>380</v>
+        <v>347</v>
       </c>
       <c r="D46" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E46" t="s">
         <v>130</v>
       </c>
       <c r="F46" t="s">
-        <v>467</v>
+        <v>450</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2763,13 +2763,13 @@
         <v>133</v>
       </c>
       <c r="D47" t="s">
-        <v>445</v>
+        <v>382</v>
       </c>
       <c r="E47" t="s">
         <v>134</v>
       </c>
       <c r="F47" t="s">
-        <v>447</v>
+        <v>475</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2780,13 +2780,13 @@
         <v>135</v>
       </c>
       <c r="D48" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E48" t="s">
         <v>136</v>
       </c>
       <c r="F48" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2794,19 +2794,19 @@
         <v>131</v>
       </c>
       <c r="B49" t="s">
-        <v>381</v>
+        <v>348</v>
       </c>
       <c r="C49" t="s">
         <v>137</v>
       </c>
       <c r="D49" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E49" t="s">
         <v>138</v>
       </c>
       <c r="F49" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2814,19 +2814,19 @@
         <v>139</v>
       </c>
       <c r="B50" t="s">
-        <v>382</v>
+        <v>349</v>
       </c>
       <c r="C50" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="D50" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E50" t="s">
         <v>140</v>
       </c>
       <c r="F50" t="s">
-        <v>350</v>
+        <v>389</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2840,13 +2840,13 @@
         <v>142</v>
       </c>
       <c r="D51" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E51" t="s">
         <v>143</v>
       </c>
       <c r="F51" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2857,16 +2857,16 @@
         <v>20</v>
       </c>
       <c r="C52" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="D52" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E52" t="s">
         <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>351</v>
+        <v>390</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2880,13 +2880,13 @@
         <v>146</v>
       </c>
       <c r="D53" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E53" t="s">
         <v>147</v>
       </c>
       <c r="F53" t="s">
-        <v>352</v>
+        <v>391</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2900,13 +2900,13 @@
         <v>150</v>
       </c>
       <c r="D54" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E54" t="s">
         <v>89</v>
       </c>
       <c r="F54" t="s">
-        <v>468</v>
+        <v>456</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2914,19 +2914,19 @@
         <v>151</v>
       </c>
       <c r="B55" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="C55" t="s">
         <v>152</v>
       </c>
       <c r="D55" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E55" t="s">
         <v>153</v>
       </c>
       <c r="F55" t="s">
-        <v>469</v>
+        <v>457</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2940,13 +2940,13 @@
         <v>155</v>
       </c>
       <c r="D56" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E56" t="s">
         <v>156</v>
       </c>
       <c r="F56" t="s">
-        <v>470</v>
+        <v>458</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2960,13 +2960,13 @@
         <v>158</v>
       </c>
       <c r="D57" t="s">
-        <v>462</v>
+        <v>445</v>
       </c>
       <c r="E57" t="s">
         <v>159</v>
       </c>
       <c r="F57" t="s">
-        <v>471</v>
+        <v>446</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2980,13 +2980,13 @@
         <v>161</v>
       </c>
       <c r="D58" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E58" t="s">
         <v>162</v>
       </c>
       <c r="F58" t="s">
-        <v>353</v>
+        <v>392</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -3000,13 +3000,13 @@
         <v>165</v>
       </c>
       <c r="D59" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E59" t="s">
         <v>166</v>
       </c>
       <c r="F59" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -3017,16 +3017,16 @@
         <v>167</v>
       </c>
       <c r="C60" t="s">
-        <v>419</v>
+        <v>362</v>
       </c>
       <c r="D60" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E60" t="s">
         <v>168</v>
       </c>
       <c r="F60" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -3034,19 +3034,19 @@
         <v>169</v>
       </c>
       <c r="B61" t="s">
-        <v>383</v>
+        <v>350</v>
       </c>
       <c r="C61" t="s">
         <v>96</v>
       </c>
       <c r="D61" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E61" t="s">
         <v>170</v>
       </c>
       <c r="F61" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -3057,16 +3057,16 @@
         <v>172</v>
       </c>
       <c r="C62" t="s">
-        <v>384</v>
+        <v>351</v>
       </c>
       <c r="D62" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E62" t="s">
         <v>173</v>
       </c>
       <c r="F62" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -3080,13 +3080,13 @@
         <v>175</v>
       </c>
       <c r="D63" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E63" t="s">
         <v>176</v>
       </c>
       <c r="F63" t="s">
-        <v>354</v>
+        <v>393</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -3100,13 +3100,13 @@
         <v>178</v>
       </c>
       <c r="D64" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E64" t="s">
         <v>179</v>
       </c>
       <c r="F64" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -3117,16 +3117,16 @@
         <v>180</v>
       </c>
       <c r="C65" t="s">
-        <v>385</v>
+        <v>352</v>
       </c>
       <c r="D65" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E65" t="s">
         <v>181</v>
       </c>
       <c r="F65" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -3137,16 +3137,16 @@
         <v>183</v>
       </c>
       <c r="C66" t="s">
-        <v>386</v>
+        <v>353</v>
       </c>
       <c r="D66" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E66" t="s">
         <v>184</v>
       </c>
       <c r="F66" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -3160,13 +3160,13 @@
         <v>187</v>
       </c>
       <c r="D67" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E67" t="s">
         <v>188</v>
       </c>
       <c r="F67" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -3180,13 +3180,13 @@
         <v>191</v>
       </c>
       <c r="D68" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E68" t="s">
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>355</v>
+        <v>394</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -3200,13 +3200,13 @@
         <v>194</v>
       </c>
       <c r="D69" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E69" t="s">
         <v>195</v>
       </c>
       <c r="F69" t="s">
-        <v>356</v>
+        <v>395</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -3220,13 +3220,13 @@
         <v>197</v>
       </c>
       <c r="D70" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E70" t="s">
         <v>198</v>
       </c>
       <c r="F70" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -3237,13 +3237,13 @@
         <v>200</v>
       </c>
       <c r="D71" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E71" t="s">
         <v>201</v>
       </c>
       <c r="F71" t="s">
-        <v>357</v>
+        <v>396</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -3254,13 +3254,13 @@
         <v>203</v>
       </c>
       <c r="D72" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E72" t="s">
         <v>204</v>
       </c>
       <c r="F72" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -3268,19 +3268,19 @@
         <v>205</v>
       </c>
       <c r="B73" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="C73" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="D73" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E73" t="s">
         <v>206</v>
       </c>
       <c r="F73" t="s">
-        <v>421</v>
+        <v>430</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -3294,13 +3294,13 @@
         <v>96</v>
       </c>
       <c r="D74" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E74" t="s">
         <v>209</v>
       </c>
       <c r="F74" t="s">
-        <v>389</v>
+        <v>408</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -3314,13 +3314,13 @@
         <v>212</v>
       </c>
       <c r="D75" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E75" t="s">
         <v>213</v>
       </c>
       <c r="F75" t="s">
-        <v>338</v>
+        <v>373</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -3328,19 +3328,19 @@
         <v>214</v>
       </c>
       <c r="B76" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C76" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="D76" t="s">
-        <v>445</v>
+        <v>382</v>
       </c>
       <c r="E76" t="s">
         <v>215</v>
       </c>
       <c r="F76" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3348,19 +3348,19 @@
         <v>214</v>
       </c>
       <c r="B77" t="s">
-        <v>390</v>
+        <v>354</v>
       </c>
       <c r="C77" t="s">
         <v>216</v>
       </c>
       <c r="D77" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E77" t="s">
         <v>217</v>
       </c>
       <c r="F77" t="s">
-        <v>358</v>
+        <v>397</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -3374,13 +3374,13 @@
         <v>220</v>
       </c>
       <c r="D78" t="s">
-        <v>462</v>
+        <v>445</v>
       </c>
       <c r="E78" t="s">
         <v>221</v>
       </c>
       <c r="F78" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -3394,13 +3394,13 @@
         <v>96</v>
       </c>
       <c r="D79" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E79" t="s">
         <v>224</v>
       </c>
       <c r="F79" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -3411,13 +3411,13 @@
         <v>226</v>
       </c>
       <c r="D80" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E80" t="s">
         <v>227</v>
       </c>
       <c r="F80" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -3431,13 +3431,13 @@
         <v>230</v>
       </c>
       <c r="D81" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E81" t="s">
         <v>231</v>
       </c>
       <c r="F81" t="s">
-        <v>480</v>
+        <v>447</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -3445,16 +3445,16 @@
         <v>228</v>
       </c>
       <c r="B82" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="D82" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E82" t="s">
         <v>232</v>
       </c>
       <c r="F82" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -3468,13 +3468,13 @@
         <v>235</v>
       </c>
       <c r="D83" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E83" t="s">
         <v>236</v>
       </c>
       <c r="F83" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -3488,13 +3488,13 @@
         <v>239</v>
       </c>
       <c r="D84" t="s">
-        <v>445</v>
+        <v>382</v>
       </c>
       <c r="E84" t="s">
         <v>240</v>
       </c>
       <c r="F84" t="s">
-        <v>482</v>
+        <v>461</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -3505,13 +3505,13 @@
         <v>242</v>
       </c>
       <c r="D85" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E85" t="s">
         <v>243</v>
       </c>
       <c r="F85" t="s">
-        <v>341</v>
+        <v>374</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -3522,16 +3522,16 @@
         <v>48</v>
       </c>
       <c r="C86" t="s">
-        <v>424</v>
+        <v>363</v>
       </c>
       <c r="D86" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E86" t="s">
         <v>244</v>
       </c>
       <c r="F86" t="s">
-        <v>483</v>
+        <v>462</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3545,13 +3545,13 @@
         <v>247</v>
       </c>
       <c r="D87" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E87" t="s">
         <v>7</v>
       </c>
       <c r="F87" t="s">
-        <v>355</v>
+        <v>394</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -3565,13 +3565,13 @@
         <v>250</v>
       </c>
       <c r="D88" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E88" t="s">
         <v>251</v>
       </c>
       <c r="F88" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -3579,16 +3579,16 @@
         <v>252</v>
       </c>
       <c r="B89" t="s">
-        <v>391</v>
+        <v>355</v>
       </c>
       <c r="D89" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E89" t="s">
         <v>253</v>
       </c>
       <c r="F89" t="s">
-        <v>359</v>
+        <v>398</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3599,16 +3599,16 @@
         <v>255</v>
       </c>
       <c r="C90" t="s">
-        <v>392</v>
+        <v>356</v>
       </c>
       <c r="D90" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E90" t="s">
         <v>256</v>
       </c>
       <c r="F90" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3619,16 +3619,16 @@
         <v>48</v>
       </c>
       <c r="C91" t="s">
-        <v>427</v>
+        <v>364</v>
       </c>
       <c r="D91" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E91" t="s">
         <v>258</v>
       </c>
       <c r="F91" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -3642,13 +3642,13 @@
         <v>261</v>
       </c>
       <c r="D92" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E92" t="s">
         <v>262</v>
       </c>
       <c r="F92" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3662,13 +3662,13 @@
         <v>265</v>
       </c>
       <c r="D93" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E93" t="s">
         <v>266</v>
       </c>
       <c r="F93" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -3682,13 +3682,13 @@
         <v>268</v>
       </c>
       <c r="D94" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E94" t="s">
         <v>269</v>
       </c>
       <c r="F94" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -3696,19 +3696,19 @@
         <v>270</v>
       </c>
       <c r="B95" t="s">
-        <v>394</v>
+        <v>357</v>
       </c>
       <c r="C95" t="s">
-        <v>360</v>
+        <v>337</v>
       </c>
       <c r="D95" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E95" t="s">
         <v>271</v>
       </c>
       <c r="F95" t="s">
-        <v>361</v>
+        <v>399</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -3716,16 +3716,16 @@
         <v>272</v>
       </c>
       <c r="B96" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D96" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E96" t="s">
         <v>273</v>
       </c>
       <c r="F96" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3736,16 +3736,16 @@
         <v>275</v>
       </c>
       <c r="C97" t="s">
-        <v>395</v>
+        <v>358</v>
       </c>
       <c r="D97" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E97" t="s">
         <v>276</v>
       </c>
       <c r="F97" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3756,13 +3756,13 @@
         <v>278</v>
       </c>
       <c r="D98" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E98" t="s">
         <v>279</v>
       </c>
       <c r="F98" t="s">
-        <v>362</v>
+        <v>400</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3770,19 +3770,19 @@
         <v>280</v>
       </c>
       <c r="B99" t="s">
-        <v>396</v>
+        <v>359</v>
       </c>
       <c r="C99" t="s">
         <v>281</v>
       </c>
       <c r="D99" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E99" t="s">
         <v>101</v>
       </c>
       <c r="F99" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3793,16 +3793,16 @@
         <v>135</v>
       </c>
       <c r="C100" t="s">
-        <v>431</v>
+        <v>365</v>
       </c>
       <c r="D100" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E100" t="s">
         <v>282</v>
       </c>
       <c r="F100" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3813,16 +3813,16 @@
         <v>283</v>
       </c>
       <c r="C101" t="s">
-        <v>433</v>
+        <v>366</v>
       </c>
       <c r="D101" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E101" t="s">
         <v>284</v>
       </c>
       <c r="F101" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3833,13 +3833,13 @@
         <v>286</v>
       </c>
       <c r="D102" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E102" t="s">
         <v>287</v>
       </c>
       <c r="F102" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -3850,13 +3850,13 @@
         <v>85</v>
       </c>
       <c r="D103" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E103" t="s">
         <v>288</v>
       </c>
       <c r="F103" t="s">
-        <v>452</v>
+        <v>487</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -3867,13 +3867,13 @@
         <v>114</v>
       </c>
       <c r="D104" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E104" t="s">
         <v>290</v>
       </c>
       <c r="F104" t="s">
-        <v>453</v>
+        <v>488</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -3884,13 +3884,13 @@
         <v>292</v>
       </c>
       <c r="D105" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E105" t="s">
         <v>293</v>
       </c>
       <c r="F105" t="s">
-        <v>363</v>
+        <v>401</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3901,16 +3901,16 @@
         <v>167</v>
       </c>
       <c r="C106" t="s">
-        <v>436</v>
+        <v>367</v>
       </c>
       <c r="D106" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E106" t="s">
         <v>295</v>
       </c>
       <c r="F106" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -3924,13 +3924,13 @@
         <v>298</v>
       </c>
       <c r="D107" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E107" t="s">
         <v>299</v>
       </c>
       <c r="F107" t="s">
-        <v>397</v>
+        <v>381</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -3944,13 +3944,13 @@
         <v>302</v>
       </c>
       <c r="D108" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E108" t="s">
         <v>303</v>
       </c>
       <c r="F108" t="s">
-        <v>454</v>
+        <v>383</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3964,13 +3964,13 @@
         <v>305</v>
       </c>
       <c r="D109" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="E109" t="s">
         <v>306</v>
       </c>
       <c r="F109" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3984,13 +3984,13 @@
         <v>96</v>
       </c>
       <c r="D110" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="E110" t="s">
         <v>309</v>
       </c>
       <c r="F110" t="s">
-        <v>486</v>
+        <v>463</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -4004,13 +4004,13 @@
         <v>310</v>
       </c>
       <c r="D111" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E111" t="s">
         <v>311</v>
       </c>
       <c r="F111" t="s">
-        <v>487</v>
+        <v>464</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -4021,16 +4021,16 @@
         <v>312</v>
       </c>
       <c r="C112" t="s">
-        <v>439</v>
+        <v>368</v>
       </c>
       <c r="D112" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="E112" t="s">
         <v>313</v>
       </c>
       <c r="F112" t="s">
-        <v>488</v>
+        <v>465</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -4041,16 +4041,16 @@
         <v>315</v>
       </c>
       <c r="C113" t="s">
-        <v>440</v>
+        <v>369</v>
       </c>
       <c r="D113" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="E113" t="s">
         <v>316</v>
       </c>
       <c r="F113" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -4061,13 +4061,13 @@
         <v>318</v>
       </c>
       <c r="D114" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="E114" t="s">
         <v>319</v>
       </c>
       <c r="F114" t="s">
-        <v>364</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>